<commit_message>
Add some prod pricing data
</commit_message>
<xml_diff>
--- a/data/product_pricing/products_data/prod_product_id_7_29-07-2026.xlsx
+++ b/data/product_pricing/products_data/prod_product_id_7_29-07-2026.xlsx
@@ -199,8 +199,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -334,225 +338,225 @@
   <dimension ref="A1:AG2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="25.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="26.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="20.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="28.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="25.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="22.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="15.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="17.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="16.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="14.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="16.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="25.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="26.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="20.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="28.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="25.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="22.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="15.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="17.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="16.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="14.93"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AG1" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="2" t="n">
         <v>17.418</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>3.65</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="2" t="n">
         <v>4.57</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G2" s="2" t="n">
         <v>1.7418</v>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>3.1</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="I2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>0.1</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K2" s="2" t="n">
         <v>4407</v>
       </c>
-      <c r="L2" s="1" t="n">
+      <c r="L2" s="2" t="n">
         <v>0.0315</v>
       </c>
-      <c r="M2" s="1" t="n">
+      <c r="M2" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="N2" s="1" t="n">
+      <c r="N2" s="2" t="n">
         <v>1611</v>
       </c>
-      <c r="O2" s="1" t="n">
+      <c r="O2" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="P2" s="1" t="n">
+      <c r="P2" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="Q2" s="1" t="n">
+      <c r="Q2" s="2" t="n">
         <v>10.93076</v>
       </c>
-      <c r="R2" s="1" t="n">
+      <c r="R2" s="2" t="n">
         <v>17.418</v>
       </c>
-      <c r="S2" s="1" t="n">
+      <c r="S2" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="T2" s="1" t="n">
+      <c r="T2" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="U2" s="1" t="n">
+      <c r="U2" s="2" t="n">
         <v>127.5</v>
       </c>
-      <c r="V2" s="1" t="n">
+      <c r="V2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="W2" s="1" t="n">
+      <c r="W2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="X2" s="1" t="n">
+      <c r="X2" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="Y2" s="1" t="n">
+      <c r="Y2" s="2" t="n">
         <v>5509800</v>
       </c>
-      <c r="Z2" s="1" t="n">
+      <c r="Z2" s="2" t="n">
         <v>76100</v>
       </c>
-      <c r="AA2" s="1" t="n">
+      <c r="AA2" s="2" t="n">
         <v>192800000</v>
       </c>
-      <c r="AB2" s="1" t="n">
+      <c r="AB2" s="2" t="n">
         <v>0.1199</v>
       </c>
-      <c r="AC2" s="1" t="n">
+      <c r="AC2" s="2" t="n">
         <v>0.0218</v>
       </c>
-      <c r="AD2" s="1" t="n">
+      <c r="AD2" s="2" t="n">
         <v>0.009</v>
       </c>
-      <c r="AE2" s="1" t="n">
+      <c r="AE2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AF2" s="1" t="n">
+      <c r="AF2" s="2" t="n">
         <v>0.08</v>
       </c>
-      <c r="AG2" s="1" t="n">
+      <c r="AG2" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>

</xml_diff>